<commit_message>
Reconcile FY 2025-26 statements to the filed ITR-5 (A.Y. 2026-27)
Every figure in the statements ties to the ITR-5 schedules: revenue
923,729; Advertisement 304,000; Telephone 3,918; other-expenses schedule
629,530 (total expenses 937,448); trade creditors 28,229; other payables
8,950; advances 409,311; bank 45,672; other cash equivalents 18,475; and
accumulated loss 13,721.

Note 9 now carries a nil "Cash on hand" line, matching the ITR-5's
distinct (blank) "Cash in hand" row, which also confirms the 18,475 sits
under "Others" within cash and cash equivalents rather than in hand.

No figure changed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157wfZAhnPBTpe9igEAtNM8
</commit_message>
<xml_diff>
--- a/Star_Fandom_India_LLP_Financial_Statements_FY_2025-26.xlsx
+++ b/Star_Fandom_India_LLP_Financial_Statements_FY_2025-26.xlsx
@@ -3831,7 +3831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:D45"/>
+  <dimension ref="B1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.6" customWidth="1" min="1" max="1"/>
@@ -4101,83 +4101,83 @@
     <row r="29" ht="13" customHeight="1">
       <c r="B29" s="14" t="inlineStr">
         <is>
+          <t>Cash on hand</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="13" customHeight="1">
+      <c r="B30" s="14" t="inlineStr">
+        <is>
           <t>Others</t>
         </is>
       </c>
-      <c r="D29" s="15" t="n">
+      <c r="D30" s="15" t="n">
         <v>18475</v>
       </c>
     </row>
-    <row r="30" ht="13" customHeight="1">
-      <c r="B30" s="55" t="inlineStr">
+    <row r="31" ht="13" customHeight="1">
+      <c r="B31" s="55" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C30" s="56" t="inlineStr">
+      <c r="C31" s="56" t="inlineStr">
         <is>
           <t>(I)</t>
         </is>
       </c>
-      <c r="D30" s="57" t="n">
+      <c r="D31" s="57" t="n">
         <v>64147</v>
       </c>
     </row>
-    <row r="31" ht="8" customHeight="1">
-      <c r="B31" s="7" t="n"/>
-      <c r="D31" s="11" t="n"/>
-    </row>
-    <row r="32" ht="13" customHeight="1">
-      <c r="B32" s="48" t="inlineStr">
+    <row r="32" ht="8" customHeight="1">
+      <c r="B32" s="7" t="n"/>
+      <c r="D32" s="11" t="n"/>
+    </row>
+    <row r="33" ht="13" customHeight="1">
+      <c r="B33" s="48" t="inlineStr">
         <is>
           <t>Other bank balances</t>
         </is>
       </c>
-      <c r="D32" s="11" t="n"/>
-    </row>
-    <row r="33" ht="13" customHeight="1">
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Bank Deposits</t>
-        </is>
-      </c>
-      <c r="D33" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="D33" s="11" t="n"/>
     </row>
     <row r="34" ht="13" customHeight="1">
       <c r="B34" s="13" t="inlineStr">
         <is>
+          <t>Bank Deposits</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="13" customHeight="1">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
           <t>Earmarked Bank Deposits</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="B35" s="50" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="B36" s="50" t="inlineStr">
         <is>
           <t>Deposits with original maturity for more than 3 months but
 less than 12 months from reporting date</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="13" customHeight="1">
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Margin money or deposits under lien</t>
-        </is>
-      </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
           <t>-</t>
@@ -4187,107 +4187,119 @@
     <row r="37" ht="13" customHeight="1">
       <c r="B37" s="13" t="inlineStr">
         <is>
+          <t>Margin money or deposits under lien</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="13" customHeight="1">
+      <c r="B38" s="13" t="inlineStr">
+        <is>
           <t>Others (specify nature)</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="13" customHeight="1">
-      <c r="B38" s="51" t="inlineStr">
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="13" customHeight="1">
+      <c r="B39" s="51" t="inlineStr">
         <is>
           <t>Total other bank balances</t>
         </is>
       </c>
-      <c r="C38" s="56" t="inlineStr">
+      <c r="C39" s="56" t="inlineStr">
         <is>
           <t>(II)</t>
         </is>
       </c>
-      <c r="D38" s="52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="13" customHeight="1">
-      <c r="B39" s="46" t="inlineStr">
+      <c r="D39" s="52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="13" customHeight="1">
+      <c r="B40" s="46" t="inlineStr">
         <is>
           <t>Total Cash and bank balances</t>
         </is>
       </c>
-      <c r="C39" s="58" t="inlineStr">
+      <c r="C40" s="58" t="inlineStr">
         <is>
           <t>(I+II)</t>
         </is>
       </c>
-      <c r="D39" s="21" t="n">
+      <c r="D40" s="21" t="n">
         <v>64147</v>
       </c>
     </row>
-    <row r="41" ht="13" customHeight="1">
-      <c r="C41" s="44" t="inlineStr">
+    <row r="42" ht="13" customHeight="1">
+      <c r="C42" s="44" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="14" customHeight="1">
-      <c r="B42" s="45" t="inlineStr">
+    <row r="43" ht="14" customHeight="1">
+      <c r="B43" s="45" t="inlineStr">
         <is>
           <t>Note 10 : Short-term loans and advances</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="28" customHeight="1">
-      <c r="B43" s="10" t="inlineStr">
+    <row r="44" ht="28" customHeight="1">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>Particulars</t>
         </is>
       </c>
-      <c r="C43" s="38" t="n"/>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="C44" s="38" t="n"/>
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>As at
 March 31, 2026</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="13" customHeight="1">
-      <c r="B44" s="13" t="inlineStr">
+    <row r="45" ht="13" customHeight="1">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>Advances</t>
         </is>
       </c>
-      <c r="D44" s="15" t="n">
+      <c r="D45" s="15" t="n">
         <v>409311</v>
       </c>
     </row>
-    <row r="45" ht="13" customHeight="1">
-      <c r="B45" s="49" t="inlineStr">
+    <row r="46" ht="13" customHeight="1">
+      <c r="B46" s="49" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C45" s="41" t="n"/>
-      <c r="D45" s="21" t="n">
+      <c r="C46" s="41" t="n"/>
+      <c r="D46" s="21" t="n">
         <v>409311</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B44:C44"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B1:D1"/>
-    <mergeCell ref="C41:D41"/>
     <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C42:D42"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B43:C43"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>